<commit_message>
Fix Maker Player TclError: resolve TCL_LIBRARY/TK_LIBRARY before tkinter import
</commit_message>
<xml_diff>
--- a/seed-files/Customer Service Alert Board 2026.xlsx
+++ b/seed-files/Customer Service Alert Board 2026.xlsx
@@ -568,7 +568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD4"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -642,7 +642,7 @@
       </c>
       <c r="B2" s="7" t="inlineStr">
         <is>
-          <t>PR TBD</t>
+          <t>Filling</t>
         </is>
       </c>
       <c r="C2" s="8" t="inlineStr">
@@ -665,10 +665,8 @@
           <t>4/23: Open PR to consume beads to avoid $$$ scrap</t>
         </is>
       </c>
-      <c r="G2" s="8" t="inlineStr">
-        <is>
-          <t>47</t>
-        </is>
+      <c r="G2" s="8" t="n">
+        <v>47</v>
       </c>
       <c r="H2" s="8" t="inlineStr">
         <is>
@@ -684,17 +682,17 @@
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>88%</t>
         </is>
       </c>
       <c r="B3" s="8" t="inlineStr">
         <is>
-          <t>Filling</t>
+          <t>Packaging</t>
         </is>
       </c>
       <c r="C3" s="8" t="inlineStr">
         <is>
-          <t>AD</t>
+          <t>JM</t>
         </is>
       </c>
       <c r="D3" s="8" t="inlineStr">
@@ -707,24 +705,18 @@
           <t>A42362</t>
         </is>
       </c>
-      <c r="F3" s="8" t="inlineStr">
-        <is>
-          <t>Extended-date lot confirmed via Teams, proceeding to production order.</t>
-        </is>
-      </c>
-      <c r="G3" s="8" t="inlineStr">
-        <is>
-          <t>18</t>
-        </is>
+      <c r="F3" s="8" t="inlineStr"/>
+      <c r="G3" s="8" t="n">
+        <v>12</v>
       </c>
       <c r="H3" s="8" t="inlineStr">
         <is>
-          <t>9/15/2026</t>
+          <t>7/2/2026</t>
         </is>
       </c>
       <c r="I3" s="9" t="inlineStr">
         <is>
-          <t>9/10/2026</t>
+          <t>7/10/2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Vendor exact Tcl/Tk 8.6.12 library, fix version-mismatch TclError via retry chain
</commit_message>
<xml_diff>
--- a/seed-files/Customer Service Alert Board 2026.xlsx
+++ b/seed-files/Customer Service Alert Board 2026.xlsx
@@ -568,7 +568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:AD4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -642,7 +642,7 @@
       </c>
       <c r="B2" s="7" t="inlineStr">
         <is>
-          <t>Filling</t>
+          <t>PR TBD</t>
         </is>
       </c>
       <c r="C2" s="8" t="inlineStr">
@@ -665,8 +665,10 @@
           <t>4/23: Open PR to consume beads to avoid $$$ scrap</t>
         </is>
       </c>
-      <c r="G2" s="8" t="n">
-        <v>47</v>
+      <c r="G2" s="8" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
       </c>
       <c r="H2" s="8" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Fix Maker Player TypeError: avoid PIL ImageTk bridge, use native tkinter.PhotoImage
</commit_message>
<xml_diff>
--- a/seed-files/Customer Service Alert Board 2026.xlsx
+++ b/seed-files/Customer Service Alert Board 2026.xlsx
@@ -568,7 +568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD4"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -642,7 +642,7 @@
       </c>
       <c r="B2" s="7" t="inlineStr">
         <is>
-          <t>PR TBD</t>
+          <t>Filling</t>
         </is>
       </c>
       <c r="C2" s="8" t="inlineStr">
@@ -665,10 +665,8 @@
           <t>4/23: Open PR to consume beads to avoid $$$ scrap</t>
         </is>
       </c>
-      <c r="G2" s="8" t="inlineStr">
-        <is>
-          <t>47</t>
-        </is>
+      <c r="G2" s="8" t="n">
+        <v>47</v>
       </c>
       <c r="H2" s="8" t="inlineStr">
         <is>

</xml_diff>